<commit_message>
prototype behuizing geprint, nu bezig met finale design
</commit_message>
<xml_diff>
--- a/Documentatie/Datasheets & Materiaal lijst/Materiaal lijst.xlsx
+++ b/Documentatie/Datasheets & Materiaal lijst/Materiaal lijst.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aaron\Desktop\PX1 - BrakeNBlink\BrakeNBlink\Documentatie\Datasheets &amp; Materiaal lijst\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA76AC1E-2E62-4D81-B13D-38AC55CCF662}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C1AC068-C849-4F25-B1A6-3C915541E8F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="66">
   <si>
     <t>drukknoppen</t>
   </si>
@@ -219,6 +219,21 @@
   </si>
   <si>
     <t>https://www.tinytronics.nl/nl/verlichting/led-strips/accessoires/jst-sm-3p-compatible-verlengkabel-30cm</t>
+  </si>
+  <si>
+    <t>Afgekeurd voor aankoop</t>
+  </si>
+  <si>
+    <t>N.v.t</t>
+  </si>
+  <si>
+    <t>Uit bestelijst exele gehaald 12/02/2026</t>
+  </si>
+  <si>
+    <t>10-pins vrouwelijke 11 mm hoge stapelbare headerconnector (OT3782)</t>
+  </si>
+  <si>
+    <t>https://www.otronic.nl/nl/10-pins-vrouwelijke-11-mm-hoge-stapelbare-headerco.html</t>
   </si>
 </sst>
 </file>
@@ -277,7 +292,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -292,6 +307,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -672,23 +690,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A2:T29"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.7265625" customWidth="1"/>
-    <col min="2" max="2" width="15.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.90625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.77734375" customWidth="1"/>
+    <col min="2" max="2" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.88671875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.36328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.08984375" customWidth="1"/>
-    <col min="9" max="9" width="10.90625" customWidth="1"/>
-    <col min="10" max="10" width="9.81640625" customWidth="1"/>
-    <col min="11" max="11" width="15.90625" customWidth="1"/>
-    <col min="12" max="12" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.109375" customWidth="1"/>
+    <col min="9" max="9" width="10.88671875" customWidth="1"/>
+    <col min="10" max="10" width="9.77734375" customWidth="1"/>
+    <col min="11" max="11" width="15.88671875" customWidth="1"/>
+    <col min="12" max="12" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="10.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:20" s="1" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:20" s="1" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>22</v>
       </c>
@@ -750,7 +769,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>7</v>
       </c>
@@ -774,7 +793,7 @@
       <c r="S3" s="3"/>
       <c r="T3" s="3"/>
     </row>
-    <row r="4" spans="1:20" ht="87" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:20" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>2</v>
       </c>
@@ -810,7 +829,7 @@
       <c r="S4" s="3"/>
       <c r="T4" s="3"/>
     </row>
-    <row r="5" spans="1:20" ht="87" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:20" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>2</v>
       </c>
@@ -820,7 +839,9 @@
         <v>0</v>
       </c>
       <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
+      <c r="F5" s="6">
+        <v>46065</v>
+      </c>
       <c r="G5" s="3">
         <v>6</v>
       </c>
@@ -845,10 +866,12 @@
       <c r="P5" s="3"/>
       <c r="Q5" s="3"/>
       <c r="R5" s="3"/>
-      <c r="S5" s="3"/>
+      <c r="S5" s="6">
+        <v>46079</v>
+      </c>
       <c r="T5" s="3"/>
     </row>
-    <row r="6" spans="1:20" ht="87" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:20" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
         <v>4</v>
       </c>
@@ -884,7 +907,7 @@
       <c r="S6" s="3"/>
       <c r="T6" s="3"/>
     </row>
-    <row r="7" spans="1:20" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:20" ht="72" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
         <v>3</v>
       </c>
@@ -892,7 +915,9 @@
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
+      <c r="F7" s="6">
+        <v>46065</v>
+      </c>
       <c r="G7" s="3">
         <v>3</v>
       </c>
@@ -920,7 +945,7 @@
       <c r="S7" s="3"/>
       <c r="T7" s="3"/>
     </row>
-    <row r="8" spans="1:20" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:20" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A8" s="3">
         <v>4</v>
       </c>
@@ -928,7 +953,9 @@
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
+      <c r="F8" s="6">
+        <v>46065</v>
+      </c>
       <c r="G8" s="3">
         <v>4</v>
       </c>
@@ -951,10 +978,12 @@
       <c r="P8" s="3"/>
       <c r="Q8" s="3"/>
       <c r="R8" s="3"/>
-      <c r="S8" s="3"/>
+      <c r="S8" s="6">
+        <v>46079</v>
+      </c>
       <c r="T8" s="3"/>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A9" s="3">
         <v>2</v>
       </c>
@@ -986,7 +1015,7 @@
       <c r="S9" s="3"/>
       <c r="T9" s="3"/>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A10" s="3">
         <v>1</v>
       </c>
@@ -1018,7 +1047,7 @@
       <c r="S10" s="3"/>
       <c r="T10" s="3"/>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A11" s="3">
         <v>2</v>
       </c>
@@ -1050,7 +1079,7 @@
       <c r="S11" s="3"/>
       <c r="T11" s="3"/>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A12" s="3">
         <v>1</v>
       </c>
@@ -1082,7 +1111,7 @@
       <c r="S12" s="3"/>
       <c r="T12" s="3"/>
     </row>
-    <row r="13" spans="1:20" ht="116" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:20" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A13" s="3">
         <v>0</v>
       </c>
@@ -1120,7 +1149,7 @@
       <c r="S13" s="3"/>
       <c r="T13" s="3"/>
     </row>
-    <row r="14" spans="1:20" ht="116" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:20" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A14" s="3">
         <v>2</v>
       </c>
@@ -1156,7 +1185,7 @@
       <c r="S14" s="3"/>
       <c r="T14" s="3"/>
     </row>
-    <row r="15" spans="1:20" ht="145" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:20" ht="144" x14ac:dyDescent="0.3">
       <c r="A15" s="3">
         <v>1</v>
       </c>
@@ -1192,17 +1221,21 @@
       <c r="S15" s="3"/>
       <c r="T15" s="3"/>
     </row>
-    <row r="16" spans="1:20" ht="145" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:20" ht="144" x14ac:dyDescent="0.3">
       <c r="A16" s="3">
         <v>1</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C16" s="3"/>
+      <c r="C16" s="3" t="s">
+        <v>61</v>
+      </c>
       <c r="D16" s="3"/>
       <c r="E16" s="3"/>
-      <c r="F16" s="3"/>
+      <c r="F16" s="6">
+        <v>46065</v>
+      </c>
       <c r="G16" s="3">
         <v>1</v>
       </c>
@@ -1225,10 +1258,12 @@
       <c r="P16" s="3"/>
       <c r="Q16" s="3"/>
       <c r="R16" s="3"/>
-      <c r="S16" s="3"/>
+      <c r="S16" s="3" t="s">
+        <v>62</v>
+      </c>
       <c r="T16" s="3"/>
     </row>
-    <row r="17" spans="1:20" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:20" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A17" s="3">
         <v>2</v>
       </c>
@@ -1264,15 +1299,19 @@
       <c r="S17" s="3"/>
       <c r="T17" s="3"/>
     </row>
-    <row r="18" spans="1:20" ht="145" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:20" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A18" s="3">
         <v>3</v>
       </c>
-      <c r="B18" s="3"/>
+      <c r="B18" s="3" t="s">
+        <v>63</v>
+      </c>
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
       <c r="E18" s="3"/>
-      <c r="F18" s="3"/>
+      <c r="F18" s="6">
+        <v>46065</v>
+      </c>
       <c r="G18" s="3">
         <v>3</v>
       </c>
@@ -1297,10 +1336,12 @@
       <c r="P18" s="3"/>
       <c r="Q18" s="3"/>
       <c r="R18" s="3"/>
-      <c r="S18" s="3"/>
+      <c r="S18" s="3" t="s">
+        <v>62</v>
+      </c>
       <c r="T18" s="3"/>
     </row>
-    <row r="19" spans="1:20" ht="116" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:20" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A19" s="3">
         <v>6</v>
       </c>
@@ -1310,7 +1351,9 @@
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
+      <c r="F19" s="6">
+        <v>46065</v>
+      </c>
       <c r="G19" s="3">
         <v>6</v>
       </c>
@@ -1333,22 +1376,34 @@
       <c r="P19" s="3"/>
       <c r="Q19" s="3"/>
       <c r="R19" s="3"/>
-      <c r="S19" s="3"/>
+      <c r="S19" s="6">
+        <v>46079</v>
+      </c>
       <c r="T19" s="3"/>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:20" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A20" s="3"/>
-      <c r="B20" s="3"/>
+      <c r="B20" s="3" t="s">
+        <v>51</v>
+      </c>
       <c r="C20" s="3"/>
       <c r="D20" s="3"/>
       <c r="E20" s="3"/>
-      <c r="F20" s="3"/>
+      <c r="F20" s="6">
+        <v>46065</v>
+      </c>
       <c r="G20" s="3"/>
-      <c r="H20" s="3"/>
+      <c r="H20" s="3" t="s">
+        <v>64</v>
+      </c>
       <c r="I20" s="3"/>
       <c r="J20" s="3"/>
-      <c r="K20" s="4"/>
-      <c r="L20" s="5"/>
+      <c r="K20" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="L20" s="5">
+        <v>12</v>
+      </c>
       <c r="M20" s="3"/>
       <c r="N20" s="3"/>
       <c r="O20" s="3"/>
@@ -1358,7 +1413,7 @@
       <c r="S20" s="3"/>
       <c r="T20" s="3"/>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A21" s="3"/>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
@@ -1380,7 +1435,7 @@
       <c r="S21" s="3"/>
       <c r="T21" s="3"/>
     </row>
-    <row r="22" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:20" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A22" s="3"/>
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
@@ -1404,7 +1459,7 @@
       <c r="S22" s="3"/>
       <c r="T22" s="3"/>
     </row>
-    <row r="23" spans="1:20" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:20" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A23" s="3">
         <v>1</v>
       </c>
@@ -1416,7 +1471,9 @@
         <v>0</v>
       </c>
       <c r="E23" s="3"/>
-      <c r="F23" s="3"/>
+      <c r="F23" s="6">
+        <v>46065</v>
+      </c>
       <c r="G23" s="3">
         <v>1</v>
       </c>
@@ -1442,7 +1499,7 @@
       <c r="S23" s="3"/>
       <c r="T23" s="3"/>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
@@ -1464,7 +1521,7 @@
       <c r="S24" s="3"/>
       <c r="T24" s="3"/>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A25" s="3"/>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
@@ -1486,7 +1543,7 @@
       <c r="S25" s="3"/>
       <c r="T25" s="3"/>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A26" s="3"/>
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
@@ -1508,7 +1565,7 @@
       <c r="S26" s="3"/>
       <c r="T26" s="3"/>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A27" s="3"/>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
@@ -1530,7 +1587,7 @@
       <c r="S27" s="3"/>
       <c r="T27" s="3"/>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A28" s="3"/>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
@@ -1552,7 +1609,7 @@
       <c r="S28" s="3"/>
       <c r="T28" s="3"/>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A29" s="3"/>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
@@ -1589,11 +1646,12 @@
     <hyperlink ref="K7" r:id="rId10" xr:uid="{E4F33FE5-5923-40B7-BC8B-C0C00E95631A}"/>
     <hyperlink ref="K18" r:id="rId11" xr:uid="{ED3872C5-9143-40BC-9373-9E0F69590981}"/>
     <hyperlink ref="K19" r:id="rId12" xr:uid="{D75B5948-5920-4534-8C2E-E90A74B3C724}"/>
+    <hyperlink ref="K20" r:id="rId13" xr:uid="{61D311D3-CA8B-4426-92A1-9418C7E9F48B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId13"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId14"/>
   <tableParts count="1">
-    <tablePart r:id="rId14"/>
+    <tablePart r:id="rId15"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Laatste controle materiaal lijst : overzicht document OK
</commit_message>
<xml_diff>
--- a/Documentatie/Datasheets & Materiaal lijst/Materiaal lijst.xlsx
+++ b/Documentatie/Datasheets & Materiaal lijst/Materiaal lijst.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aaron\Desktop\PX1 - BrakeNBlink\BrakeNBlink\Documentatie\Datasheets &amp; Materiaal lijst\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B84E0920-251D-4167-95C1-D7B15AAF40A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0512F1D1-81DF-46C5-967B-A0DF3CEC4668}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -370,7 +370,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -395,9 +395,6 @@
     </xf>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -439,7 +436,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -455,19 +452,19 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FF0E2E08-0CB4-41D1-909A-9866F9E2FAC5}" name="Tabel1" displayName="Tabel1" ref="A2:J53" totalsRowShown="0" headerRowDxfId="11" dataDxfId="0">
-  <autoFilter ref="A2:J53" xr:uid="{FF0E2E08-0CB4-41D1-909A-9866F9E2FAC5}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FF0E2E08-0CB4-41D1-909A-9866F9E2FAC5}" name="Tabel1" displayName="Tabel1" ref="A2:J49" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+  <autoFilter ref="A2:J49" xr:uid="{FF0E2E08-0CB4-41D1-909A-9866F9E2FAC5}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{1B5DBAEF-1276-450F-A9EA-3F4E61E1B2D4}" name="Aantal nodig" dataDxfId="10"/>
-    <tableColumn id="20" xr3:uid="{B5B5338E-5671-42DF-BCC5-235E2DA36C6E}" name="Datasheets OK" dataDxfId="9"/>
-    <tableColumn id="18" xr3:uid="{76C77F8A-EF04-4113-8E13-24A5F4207CBE}" name="Op school" dataDxfId="8"/>
-    <tableColumn id="8" xr3:uid="{8B66298D-DF14-4969-A852-7F6A53B8671A}" name="aantal te kopen" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{A4DC773C-F033-4DA0-AA0D-B21739089B2C}" name="Korte omschrijving" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{80982AC6-7BD3-4773-8CEC-D400BD08E6CB}" name="winkel" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{DF4EED70-3D1C-446A-91B1-86731E303698}" name="artikelnummer" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{8EF30C82-0B38-42F2-A1A5-6BB9095E8F15}" name="Url" dataDxfId="3"/>
-    <tableColumn id="15" xr3:uid="{5DE6143D-3D33-4B5A-AFC0-B70BB8C2156F}" name="bestelling ontvangen" dataDxfId="2"/>
-    <tableColumn id="16" xr3:uid="{26B2E2E1-82AB-46B3-A25C-EEEBCE8B8487}" name="opmerkingen" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{1B5DBAEF-1276-450F-A9EA-3F4E61E1B2D4}" name="Aantal nodig" dataDxfId="11"/>
+    <tableColumn id="20" xr3:uid="{B5B5338E-5671-42DF-BCC5-235E2DA36C6E}" name="Datasheets OK" dataDxfId="10"/>
+    <tableColumn id="18" xr3:uid="{76C77F8A-EF04-4113-8E13-24A5F4207CBE}" name="Op school" dataDxfId="9"/>
+    <tableColumn id="8" xr3:uid="{8B66298D-DF14-4969-A852-7F6A53B8671A}" name="aantal te kopen" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{A4DC773C-F033-4DA0-AA0D-B21739089B2C}" name="Korte omschrijving" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{80982AC6-7BD3-4773-8CEC-D400BD08E6CB}" name="winkel" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{DF4EED70-3D1C-446A-91B1-86731E303698}" name="artikelnummer" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{8EF30C82-0B38-42F2-A1A5-6BB9095E8F15}" name="Url" dataDxfId="4"/>
+    <tableColumn id="15" xr3:uid="{5DE6143D-3D33-4B5A-AFC0-B70BB8C2156F}" name="bestelling ontvangen" dataDxfId="3"/>
+    <tableColumn id="16" xr3:uid="{26B2E2E1-82AB-46B3-A25C-EEEBCE8B8487}" name="opmerkingen" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -752,34 +749,34 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:10" s="1" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="H2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="I2" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="J2" s="3" t="s">
         <v>9</v>
       </c>
     </row>
@@ -1476,13 +1473,13 @@
       <c r="J31" s="3"/>
     </row>
     <row r="32" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A32" s="9">
+      <c r="A32" s="3">
         <v>3</v>
       </c>
-      <c r="B32" s="9" t="s">
+      <c r="B32" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="C32" s="9" t="s">
+      <c r="C32" s="3" t="s">
         <v>70</v>
       </c>
       <c r="D32" s="3">

</xml_diff>